<commit_message>
Camas libres en consulta
</commit_message>
<xml_diff>
--- a/app/uploads/Prueba para subir excel reducido.xlsx
+++ b/app/uploads/Prueba para subir excel reducido.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="36">
   <si>
     <t>planta</t>
   </si>
@@ -109,13 +109,31 @@
   </si>
   <si>
     <t>Mary</t>
+  </si>
+  <si>
+    <t>Juan</t>
+  </si>
+  <si>
+    <t>Cabezas</t>
+  </si>
+  <si>
+    <t>Mingorance</t>
+  </si>
+  <si>
+    <t>409A</t>
+  </si>
+  <si>
+    <t>1-A-5-3-Cama3</t>
+  </si>
+  <si>
+    <t>OCUpada</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,6 +143,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -167,11 +193,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -476,13 +503,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="15.7109375" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -618,6 +646,53 @@
         <v>2</v>
       </c>
     </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D4">
+        <v>401</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J4">
+        <v>1</v>
+      </c>
+      <c r="K4" t="s">
+        <v>7</v>
+      </c>
+      <c r="L4">
+        <v>5</v>
+      </c>
+      <c r="M4">
+        <v>3</v>
+      </c>
+      <c r="N4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L14" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>